<commit_message>
Examples to test survey import with add / update values
</commit_message>
<xml_diff>
--- a/Examples/survey789.xlsx
+++ b/Examples/survey789.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t xml:space="preserve">Case</t>
   </si>
@@ -34,7 +34,10 @@
     <t xml:space="preserve">Interest</t>
   </si>
   <si>
-    <t xml:space="preserve">freetext</t>
+    <t xml:space="preserve">Qual_hobby_opinions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qual_pet_opinions</t>
   </si>
   <si>
     <t xml:space="preserve">ID7</t>
@@ -46,7 +49,10 @@
     <t xml:space="preserve">surveys</t>
   </si>
   <si>
-    <t xml:space="preserve">I work for a survey company, and I survey people on all kinds of topics</t>
+    <t xml:space="preserve">I work for a survey company, and I survey people on all kinds of topics. I enjoy surveys even as a hobby.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I had a pet sheepdog growing up that would sit with me for ages while I did my homework. The safety aspect is important too, nobody messes with a house that has a loud dog bark coming from inside.</t>
   </si>
   <si>
     <t xml:space="preserve">ID8</t>
@@ -61,6 +67,9 @@
     <t xml:space="preserve">I like tv programs, and my favourites are morning shows and the news</t>
   </si>
   <si>
+    <t xml:space="preserve">A fish</t>
+  </si>
+  <si>
     <t xml:space="preserve">ID9</t>
   </si>
   <si>
@@ -68,6 +77,9 @@
   </si>
   <si>
     <t xml:space="preserve">I like to read and see lots of information about economics, the area excites me, as I am an accountant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cats are the best pets,soft and cute. Dogs are needy, not bright, sometimes aggressive. Cats are laid back relaxed and sleep a lot. They are loving but not overly attention seeking. They do not require lots other than food and litter box cleaning, and the yearly vet visit.</t>
   </si>
 </sst>
 </file>
@@ -142,13 +154,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -171,37 +187,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -274,14 +290,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="4.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="6.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="109.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="25.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="27.87"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -300,53 +317,65 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>33</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="E2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>55</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>